<commit_message>
assume the commit message is "Update oversigt_over_gartnerierne.xlsx with latest data"
</commit_message>
<xml_diff>
--- a/Gartnerier i Brabrand/oversigt_over_gartnerierne.xlsx
+++ b/Gartnerier i Brabrand/oversigt_over_gartnerierne.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erikl\Documents\GitHub\Gartnerier-i-Brabrand\Gartnerier i Brabrand\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GIS\Github Update\Gartnerier-i-Brabrand\Gartnerier i Brabrand\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{519E4333-AE0E-46B9-A654-31D1122E7BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A8C320F-30A8-4EB2-A352-AEAC9F266CDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C4A0B6AA-D64C-40C5-A9A2-780F03B91B71}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{C4A0B6AA-D64C-40C5-A9A2-780F03B91B71}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="361">
   <si>
     <t>Ejer</t>
   </si>
@@ -1116,6 +1116,9 @@
   </si>
   <si>
     <t>56.161302, 10.109074</t>
+  </si>
+  <si>
+    <t>56.183684, 10.130028</t>
   </si>
 </sst>
 </file>
@@ -1548,21 +1551,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9410E6E1-B6FD-499D-B70E-01FA93ABCF11}">
   <dimension ref="A1:K103"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="14.81640625" customWidth="1"/>
-    <col min="3" max="3" width="26.54296875" customWidth="1"/>
-    <col min="4" max="4" width="28.1796875" customWidth="1"/>
-    <col min="5" max="5" width="17.26953125" customWidth="1"/>
+    <col min="1" max="2" width="14.85546875" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" customWidth="1"/>
+    <col min="4" max="4" width="28.140625" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" customWidth="1"/>
     <col min="6" max="6" width="23" customWidth="1"/>
-    <col min="7" max="7" width="21.54296875" style="9" customWidth="1"/>
-    <col min="8" max="8" width="25.1796875" customWidth="1"/>
-    <col min="9" max="9" width="25.7265625" customWidth="1"/>
-    <col min="10" max="10" width="17.81640625" customWidth="1"/>
-    <col min="11" max="11" width="36.1796875" customWidth="1"/>
+    <col min="7" max="7" width="21.5703125" style="9" customWidth="1"/>
+    <col min="8" max="8" width="25.140625" customWidth="1"/>
+    <col min="9" max="9" width="25.7109375" customWidth="1"/>
+    <col min="10" max="10" width="17.85546875" customWidth="1"/>
+    <col min="11" max="11" width="36.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -1597,7 +1600,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1626,7 +1629,7 @@
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1645,7 +1648,7 @@
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1664,7 +1667,7 @@
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1689,7 +1692,7 @@
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1716,7 +1719,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -1747,7 +1750,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1768,7 +1771,7 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1797,7 +1800,7 @@
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1826,7 +1829,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>10</v>
       </c>
@@ -1853,7 +1856,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>11</v>
       </c>
@@ -1880,7 +1883,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>12</v>
       </c>
@@ -1905,7 +1908,7 @@
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1932,7 +1935,7 @@
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1957,7 +1960,7 @@
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1982,7 +1985,7 @@
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -2007,7 +2010,7 @@
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>17</v>
       </c>
@@ -2032,7 +2035,7 @@
       <c r="J18" s="5"/>
       <c r="K18" s="5"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -2057,7 +2060,7 @@
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -2082,7 +2085,7 @@
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -2107,7 +2110,7 @@
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -2134,7 +2137,7 @@
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -2158,7 +2161,7 @@
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -2187,7 +2190,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -2216,7 +2219,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -2237,7 +2240,7 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
         <v>26</v>
       </c>
@@ -2260,7 +2263,7 @@
       <c r="J27" s="5"/>
       <c r="K27" s="5"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -2289,7 +2292,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -2314,7 +2317,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -2341,7 +2344,7 @@
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -2368,7 +2371,7 @@
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -2393,7 +2396,7 @@
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -2422,7 +2425,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -2447,7 +2450,7 @@
       <c r="J34" s="1"/>
       <c r="K34" s="1"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -2476,7 +2479,7 @@
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2497,7 +2500,7 @@
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -2524,7 +2527,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -2549,7 +2552,7 @@
       <c r="J38" s="1"/>
       <c r="K38" s="1"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -2574,7 +2577,7 @@
       <c r="J39" s="1"/>
       <c r="K39" s="1"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -2599,7 +2602,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -2630,7 +2633,7 @@
         <v>7716</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -2655,7 +2658,7 @@
         <v>6800</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -2680,7 +2683,7 @@
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -2707,7 +2710,7 @@
       <c r="J44" s="1"/>
       <c r="K44" s="1"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -2732,7 +2735,7 @@
       <c r="J45" s="1"/>
       <c r="K45" s="1"/>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -2753,7 +2756,7 @@
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -2778,7 +2781,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -2807,7 +2810,7 @@
       <c r="J48" s="1"/>
       <c r="K48" s="1"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -2832,7 +2835,7 @@
       <c r="J49" s="1"/>
       <c r="K49" s="1"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -2857,7 +2860,7 @@
       <c r="J50" s="1"/>
       <c r="K50" s="1"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
         <v>50</v>
       </c>
@@ -2882,7 +2885,7 @@
       <c r="J51" s="5"/>
       <c r="K51" s="5"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -2907,7 +2910,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -2932,7 +2935,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -2957,7 +2960,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -2982,7 +2985,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -3007,7 +3010,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>56</v>
       </c>
@@ -3030,7 +3033,7 @@
       <c r="J57" s="1"/>
       <c r="K57" s="1"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>57</v>
       </c>
@@ -3057,7 +3060,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>58</v>
       </c>
@@ -3082,7 +3085,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -3101,7 +3104,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -3126,7 +3129,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -3149,7 +3152,7 @@
       <c r="J62" s="1"/>
       <c r="K62" s="1"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -3170,7 +3173,7 @@
       <c r="J63" s="1"/>
       <c r="K63" s="1"/>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>63</v>
       </c>
@@ -3191,7 +3194,7 @@
       <c r="J64" s="1"/>
       <c r="K64" s="1"/>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>64</v>
       </c>
@@ -3216,7 +3219,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>65</v>
       </c>
@@ -3243,7 +3246,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>66</v>
       </c>
@@ -3268,7 +3271,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>67</v>
       </c>
@@ -3293,7 +3296,7 @@
       <c r="J68" s="1"/>
       <c r="K68" s="1"/>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -3316,7 +3319,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -3337,7 +3340,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>70</v>
       </c>
@@ -3362,7 +3365,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>71</v>
       </c>
@@ -3387,7 +3390,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>72</v>
       </c>
@@ -3412,7 +3415,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>73</v>
       </c>
@@ -3437,7 +3440,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>74</v>
       </c>
@@ -3458,7 +3461,7 @@
       <c r="J75" s="1"/>
       <c r="K75" s="1"/>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>75</v>
       </c>
@@ -3483,7 +3486,7 @@
       <c r="J76" s="1"/>
       <c r="K76" s="1"/>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>76</v>
       </c>
@@ -3508,7 +3511,7 @@
       <c r="J77" s="1"/>
       <c r="K77" s="1"/>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>77</v>
       </c>
@@ -3537,7 +3540,7 @@
       <c r="J78" s="1"/>
       <c r="K78" s="1"/>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>78</v>
       </c>
@@ -3560,7 +3563,7 @@
       <c r="J79" s="1"/>
       <c r="K79" s="1"/>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>79</v>
       </c>
@@ -3585,7 +3588,7 @@
       <c r="J80" s="1"/>
       <c r="K80" s="1"/>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -3610,7 +3613,7 @@
       <c r="J81" s="2"/>
       <c r="K81" s="2"/>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>81</v>
       </c>
@@ -3637,7 +3640,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>82</v>
       </c>
@@ -3658,7 +3661,7 @@
       <c r="J83" s="1"/>
       <c r="K83" s="1"/>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>83</v>
       </c>
@@ -3679,7 +3682,7 @@
       <c r="J84" s="1"/>
       <c r="K84" s="1"/>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>84</v>
       </c>
@@ -3693,14 +3696,16 @@
       <c r="E85" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="F85" s="1"/>
+      <c r="F85" s="1" t="s">
+        <v>360</v>
+      </c>
       <c r="G85" s="6"/>
       <c r="H85" s="1"/>
       <c r="I85" s="1"/>
       <c r="J85" s="1"/>
       <c r="K85" s="1"/>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>85</v>
       </c>
@@ -3727,7 +3732,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>86</v>
       </c>
@@ -3754,7 +3759,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>87</v>
       </c>
@@ -3777,7 +3782,7 @@
       <c r="J88" s="1"/>
       <c r="K88" s="1"/>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>88</v>
       </c>
@@ -3808,7 +3813,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>89</v>
       </c>
@@ -3837,7 +3842,7 @@
       <c r="J90" s="1"/>
       <c r="K90" s="1"/>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>90</v>
       </c>
@@ -3862,7 +3867,7 @@
       <c r="J91" s="1"/>
       <c r="K91" s="1"/>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>91</v>
       </c>
@@ -3885,7 +3890,7 @@
       <c r="J92" s="1"/>
       <c r="K92" s="1"/>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>92</v>
       </c>
@@ -3910,7 +3915,7 @@
       <c r="J93" s="1"/>
       <c r="K93" s="1"/>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>93</v>
       </c>
@@ -3935,7 +3940,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>94</v>
       </c>
@@ -3960,7 +3965,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>95</v>
       </c>
@@ -3987,7 +3992,7 @@
       <c r="J96" s="1"/>
       <c r="K96" s="1"/>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>96</v>
       </c>
@@ -4012,7 +4017,7 @@
       <c r="J97" s="1"/>
       <c r="K97" s="1"/>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>97</v>
       </c>
@@ -4039,7 +4044,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>98</v>
       </c>
@@ -4064,7 +4069,7 @@
       <c r="J99" s="1"/>
       <c r="K99" s="1"/>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>99</v>
       </c>
@@ -4089,7 +4094,7 @@
       <c r="J100" s="1"/>
       <c r="K100" s="1"/>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>100</v>
       </c>
@@ -4106,7 +4111,7 @@
       <c r="J101" s="1"/>
       <c r="K101" s="1"/>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>101</v>
       </c>
@@ -4121,7 +4126,7 @@
       <c r="J102" s="1"/>
       <c r="K102" s="1"/>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A103" s="1"/>
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>

</xml_diff>